<commit_message>
Plan Hamburguesería Smash: regenerados los 4 entregables y la Guía de Equivalencias (matriz con 59 productos ES)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XC64Aa7enUEgrbksa2cneQ
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-hamburgueseria/calculadora-carne-patatas-escandallo-hamburgueseria.xlsx
+++ b/astro-site/public/dl/plan-negocio-hamburgueseria/calculadora-carne-patatas-escandallo-hamburgueseria.xlsx
@@ -618,7 +618,7 @@
     <row r="3" ht="64" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>AVISO FIJO. Carne picada (RD 1021/2022, arts. 4.1, 7.2 y 7.3): comprada picada o picada en el local, se conserva a 2 °C o menos; la bola salada antes de la plancha es un preparado de carne, a 4 °C o menos; la picada en el local es del día y nunca de un día para otro. Nada de carne madurada más de 15 días (Inf26008). Los minutos de limpiar y picar (6) y la merma de cocción no tienen fuente: mídelos.</t>
+          <t>AVISO FIJO. Carne picada (RD 1021/2022, arts. 4.1, 7.2 y 7.3): comprada picada o picada en el local, se conserva a 2 °C o menos; la bola salada antes de la plancha es un preparado de carne, a 4 °C o menos; la picada en el local es del día y nunca de un día para otro. La carne madurada semanas queda fuera del plazo de picado de 6 días desde el sacrificio (15 si es vacuno al vacío) (Inf26008). Los minutos de limpiar y picar (6) y la merma de cocción no tienen fuente: mídelos.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>RD 1021/2022, arts. 7.2 y 7.3: la carne que picas en el local es del día y nunca de un día para otro; músculo sin recortes, con como máximo 6 días desde el sacrificio o 15 si va envasada al vacío. Nada de carne madurada más de 15 días (Inf26008).</t>
+          <t>RD 1021/2022, arts. 7.2 y 7.3: la carne que picas en el local es del día y nunca de un día para otro; músculo sin recortes, con como máximo 6 días desde el sacrificio o 15 si va envasada al vacío. La carne madurada semanas queda fuera de ese plazo (Inf26008).</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
     <row r="10" ht="75" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5. Carne picada (RD 1021/2022, arts. 4.1, 7.2 y 7.3). Comprada picada o picada en el local, se conserva a 2 °C o menos; la bola salada antes de la plancha es un preparado de carne, a 4 °C o menos; la picada en el local es del día y nunca de un día para otro, con músculo sin recortes y como máximo 6 días desde el sacrificio, o 15 si va envasada al vacío. Nada de carne madurada más de 15 días (Inf26008). El desplegable de la hoja es solo un recordatorio: no cambia ningún cálculo.</t>
+          <t>5. Carne picada (RD 1021/2022, arts. 4.1, 7.2 y 7.3). Comprada picada o picada en el local, se conserva a 2 °C o menos; la bola salada antes de la plancha es un preparado de carne, a 4 °C o menos; la picada en el local es del día y nunca de un día para otro, con músculo sin recortes y como máximo 6 días desde el sacrificio, o 15 si va envasada al vacío. La carne madurada semanas queda fuera de ese plazo (Inf26008). El desplegable de la hoja es solo un recordatorio: no cambia ningún cálculo.</t>
         </is>
       </c>
     </row>

</xml_diff>